<commit_message>
upload other sites case study
</commit_message>
<xml_diff>
--- a/sitkana/Fixed Vessel Cases/Site 1 Optimal/results_df.xlsx
+++ b/sitkana/Fixed Vessel Cases/Site 1 Optimal/results_df.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T298"/>
+  <dimension ref="A1:T277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17642,1308 +17642,6 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="278">
-      <c r="A278" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="B278" t="n">
-        <v>20000</v>
-      </c>
-      <c r="C278" t="n">
-        <v>14</v>
-      </c>
-      <c r="D278" t="n">
-        <v>12.99559113215011</v>
-      </c>
-      <c r="E278" t="n">
-        <v>10.0402636072274</v>
-      </c>
-      <c r="F278" t="n">
-        <v>14</v>
-      </c>
-      <c r="G278" t="n">
-        <v>7630.292013796412</v>
-      </c>
-      <c r="H278" t="n">
-        <v>0.04355189505591559</v>
-      </c>
-      <c r="I278" t="n">
-        <v>14</v>
-      </c>
-      <c r="J278" t="n">
-        <v>23.15734126984127</v>
-      </c>
-      <c r="K278" t="n">
-        <v>6209.560000000001</v>
-      </c>
-      <c r="L278" t="n">
-        <v>19496.07069700147</v>
-      </c>
-      <c r="M278" t="n">
-        <v>7655.686525581573</v>
-      </c>
-      <c r="N278" t="n">
-        <v>1490.202744702</v>
-      </c>
-      <c r="O278" t="n">
-        <v>11182.8279696</v>
-      </c>
-      <c r="P278" t="n">
-        <v>48914.13986199999</v>
-      </c>
-      <c r="Q278" t="n">
-        <v>1242.01</v>
-      </c>
-      <c r="R278" t="n">
-        <v>1542.52</v>
-      </c>
-      <c r="S278" t="n">
-        <v>350.0350000000004</v>
-      </c>
-      <c r="T278" t="n">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="279">
-      <c r="A279" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="B279" t="n">
-        <v>5000</v>
-      </c>
-      <c r="C279" t="n">
-        <v>18</v>
-      </c>
-      <c r="D279" t="n">
-        <v>9.862366503899541</v>
-      </c>
-      <c r="E279" t="n">
-        <v>9.293565808940587</v>
-      </c>
-      <c r="F279" t="n">
-        <v>14</v>
-      </c>
-      <c r="G279" t="n">
-        <v>7630.292013796412</v>
-      </c>
-      <c r="H279" t="n">
-        <v>0.1742075802236624</v>
-      </c>
-      <c r="I279" t="n">
-        <v>14</v>
-      </c>
-      <c r="J279" t="n">
-        <v>23.15734126984127</v>
-      </c>
-      <c r="K279" t="n">
-        <v>2891.56</v>
-      </c>
-      <c r="L279" t="n">
-        <v>11761.96926324595</v>
-      </c>
-      <c r="M279" t="n">
-        <v>5319.413731221542</v>
-      </c>
-      <c r="N279" t="n">
-        <v>374.4457123995</v>
-      </c>
-      <c r="O279" t="n">
-        <v>4606.35457485</v>
-      </c>
-      <c r="P279" t="n">
-        <v>16031.772862</v>
-      </c>
-      <c r="Q279" t="n">
-        <v>1242.01</v>
-      </c>
-      <c r="R279" t="n">
-        <v>1542.52</v>
-      </c>
-      <c r="S279" t="n">
-        <v>350.0350000000004</v>
-      </c>
-      <c r="T279" t="n">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="280">
-      <c r="A280" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="B280" t="n">
-        <v>20000</v>
-      </c>
-      <c r="C280" t="n">
-        <v>10</v>
-      </c>
-      <c r="D280" t="n">
-        <v>9.282565094392938</v>
-      </c>
-      <c r="E280" t="n">
-        <v>10.0402636072274</v>
-      </c>
-      <c r="F280" t="n">
-        <v>14</v>
-      </c>
-      <c r="G280" t="n">
-        <v>7630.292013796412</v>
-      </c>
-      <c r="H280" t="n">
-        <v>0.04355189505591559</v>
-      </c>
-      <c r="I280" t="n">
-        <v>14</v>
-      </c>
-      <c r="J280" t="n">
-        <v>23.15734126984127</v>
-      </c>
-      <c r="K280" t="n">
-        <v>6209.560000000001</v>
-      </c>
-      <c r="L280" t="n">
-        <v>19496.07069700147</v>
-      </c>
-      <c r="M280" t="n">
-        <v>7655.686525581573</v>
-      </c>
-      <c r="N280" t="n">
-        <v>1490.202744702</v>
-      </c>
-      <c r="O280" t="n">
-        <v>11182.8279696</v>
-      </c>
-      <c r="P280" t="n">
-        <v>48914.13986199999</v>
-      </c>
-      <c r="Q280" t="n">
-        <v>1242.01</v>
-      </c>
-      <c r="R280" t="n">
-        <v>1542.52</v>
-      </c>
-      <c r="S280" t="n">
-        <v>350.0350000000004</v>
-      </c>
-      <c r="T280" t="n">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="281">
-      <c r="A281" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="B281" t="n">
-        <v>1000</v>
-      </c>
-      <c r="C281" t="n">
-        <v>18</v>
-      </c>
-      <c r="D281" t="n">
-        <v>2.914967211530838</v>
-      </c>
-      <c r="E281" t="n">
-        <v>9.856935437888509</v>
-      </c>
-      <c r="F281" t="n">
-        <v>14</v>
-      </c>
-      <c r="G281" t="n">
-        <v>7630.292013796412</v>
-      </c>
-      <c r="H281" t="n">
-        <v>0.8710379011183119</v>
-      </c>
-      <c r="I281" t="n">
-        <v>14</v>
-      </c>
-      <c r="J281" t="n">
-        <v>23.15734126984127</v>
-      </c>
-      <c r="K281" t="n">
-        <v>2006.76</v>
-      </c>
-      <c r="L281" t="n">
-        <v>2782.955559373141</v>
-      </c>
-      <c r="M281" t="n">
-        <v>2607.085011948757</v>
-      </c>
-      <c r="N281" t="n">
-        <v>83.98837288254001</v>
-      </c>
-      <c r="O281" t="n">
-        <v>2384.207646674</v>
-      </c>
-      <c r="P281" t="n">
-        <v>4921.03817688</v>
-      </c>
-      <c r="Q281" t="n">
-        <v>1242.01</v>
-      </c>
-      <c r="R281" t="n">
-        <v>1542.52</v>
-      </c>
-      <c r="S281" t="n">
-        <v>350.0350000000004</v>
-      </c>
-      <c r="T281" t="n">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="282">
-      <c r="A282" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="B282" t="n">
-        <v>10000</v>
-      </c>
-      <c r="C282" t="n">
-        <v>10</v>
-      </c>
-      <c r="D282" t="n">
-        <v>7.853307313798277</v>
-      </c>
-      <c r="E282" t="n">
-        <v>9.591210385276415</v>
-      </c>
-      <c r="F282" t="n">
-        <v>14</v>
-      </c>
-      <c r="G282" t="n">
-        <v>7630.292013796412</v>
-      </c>
-      <c r="H282" t="n">
-        <v>0.08710379011183118</v>
-      </c>
-      <c r="I282" t="n">
-        <v>14</v>
-      </c>
-      <c r="J282" t="n">
-        <v>23.15734126984127</v>
-      </c>
-      <c r="K282" t="n">
-        <v>3997.56</v>
-      </c>
-      <c r="L282" t="n">
-        <v>15629.01998012371</v>
-      </c>
-      <c r="M282" t="n">
-        <v>6487.550128401559</v>
-      </c>
-      <c r="N282" t="n">
-        <v>741.7082303399999</v>
-      </c>
-      <c r="O282" t="n">
-        <v>7106.6838794</v>
-      </c>
-      <c r="P282" t="n">
-        <v>28533.419418</v>
-      </c>
-      <c r="Q282" t="n">
-        <v>1242.01</v>
-      </c>
-      <c r="R282" t="n">
-        <v>1542.52</v>
-      </c>
-      <c r="S282" t="n">
-        <v>350.0350000000004</v>
-      </c>
-      <c r="T282" t="n">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="283">
-      <c r="A283" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="B283" t="n">
-        <v>5000</v>
-      </c>
-      <c r="C283" t="n">
-        <v>4</v>
-      </c>
-      <c r="D283" t="n">
-        <v>2.191637000866565</v>
-      </c>
-      <c r="E283" t="n">
-        <v>9.293565808940587</v>
-      </c>
-      <c r="F283" t="n">
-        <v>14</v>
-      </c>
-      <c r="G283" t="n">
-        <v>7630.292013796412</v>
-      </c>
-      <c r="H283" t="n">
-        <v>0.1742075802236624</v>
-      </c>
-      <c r="I283" t="n">
-        <v>14</v>
-      </c>
-      <c r="J283" t="n">
-        <v>23.15734126984127</v>
-      </c>
-      <c r="K283" t="n">
-        <v>2891.56</v>
-      </c>
-      <c r="L283" t="n">
-        <v>11761.96926324595</v>
-      </c>
-      <c r="M283" t="n">
-        <v>5319.413731221542</v>
-      </c>
-      <c r="N283" t="n">
-        <v>374.4457123995</v>
-      </c>
-      <c r="O283" t="n">
-        <v>4606.35457485</v>
-      </c>
-      <c r="P283" t="n">
-        <v>16031.772862</v>
-      </c>
-      <c r="Q283" t="n">
-        <v>1242.01</v>
-      </c>
-      <c r="R283" t="n">
-        <v>1542.52</v>
-      </c>
-      <c r="S283" t="n">
-        <v>350.0350000000004</v>
-      </c>
-      <c r="T283" t="n">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="284">
-      <c r="A284" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="B284" t="n">
-        <v>1000</v>
-      </c>
-      <c r="C284" t="n">
-        <v>14</v>
-      </c>
-      <c r="D284" t="n">
-        <v>2.267196720079541</v>
-      </c>
-      <c r="E284" t="n">
-        <v>9.856935437888509</v>
-      </c>
-      <c r="F284" t="n">
-        <v>14</v>
-      </c>
-      <c r="G284" t="n">
-        <v>7630.292013796412</v>
-      </c>
-      <c r="H284" t="n">
-        <v>0.8710379011183119</v>
-      </c>
-      <c r="I284" t="n">
-        <v>14</v>
-      </c>
-      <c r="J284" t="n">
-        <v>23.15734126984127</v>
-      </c>
-      <c r="K284" t="n">
-        <v>2006.76</v>
-      </c>
-      <c r="L284" t="n">
-        <v>2782.955559373141</v>
-      </c>
-      <c r="M284" t="n">
-        <v>2607.085011948757</v>
-      </c>
-      <c r="N284" t="n">
-        <v>83.98837288254001</v>
-      </c>
-      <c r="O284" t="n">
-        <v>2384.207646674</v>
-      </c>
-      <c r="P284" t="n">
-        <v>4921.03817688</v>
-      </c>
-      <c r="Q284" t="n">
-        <v>1242.01</v>
-      </c>
-      <c r="R284" t="n">
-        <v>1542.52</v>
-      </c>
-      <c r="S284" t="n">
-        <v>350.0350000000004</v>
-      </c>
-      <c r="T284" t="n">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="285">
-      <c r="A285" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="B285" t="n">
-        <v>1000</v>
-      </c>
-      <c r="C285" t="n">
-        <v>4</v>
-      </c>
-      <c r="D285" t="n">
-        <v>0.6477704914512973</v>
-      </c>
-      <c r="E285" t="n">
-        <v>9.856935437888509</v>
-      </c>
-      <c r="F285" t="n">
-        <v>14</v>
-      </c>
-      <c r="G285" t="n">
-        <v>7630.292013796412</v>
-      </c>
-      <c r="H285" t="n">
-        <v>0.8710379011183119</v>
-      </c>
-      <c r="I285" t="n">
-        <v>14</v>
-      </c>
-      <c r="J285" t="n">
-        <v>23.15734126984127</v>
-      </c>
-      <c r="K285" t="n">
-        <v>2006.76</v>
-      </c>
-      <c r="L285" t="n">
-        <v>2782.955559373141</v>
-      </c>
-      <c r="M285" t="n">
-        <v>2607.085011948757</v>
-      </c>
-      <c r="N285" t="n">
-        <v>83.98837288254001</v>
-      </c>
-      <c r="O285" t="n">
-        <v>2384.207646674</v>
-      </c>
-      <c r="P285" t="n">
-        <v>4921.03817688</v>
-      </c>
-      <c r="Q285" t="n">
-        <v>1242.01</v>
-      </c>
-      <c r="R285" t="n">
-        <v>1542.52</v>
-      </c>
-      <c r="S285" t="n">
-        <v>350.0350000000004</v>
-      </c>
-      <c r="T285" t="n">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="286">
-      <c r="A286" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="B286" t="n">
-        <v>1000</v>
-      </c>
-      <c r="C286" t="n">
-        <v>6</v>
-      </c>
-      <c r="D286" t="n">
-        <v>0.9716557371769459</v>
-      </c>
-      <c r="E286" t="n">
-        <v>9.856935437888509</v>
-      </c>
-      <c r="F286" t="n">
-        <v>14</v>
-      </c>
-      <c r="G286" t="n">
-        <v>7630.292013796412</v>
-      </c>
-      <c r="H286" t="n">
-        <v>0.8710379011183119</v>
-      </c>
-      <c r="I286" t="n">
-        <v>14</v>
-      </c>
-      <c r="J286" t="n">
-        <v>23.15734126984127</v>
-      </c>
-      <c r="K286" t="n">
-        <v>2006.76</v>
-      </c>
-      <c r="L286" t="n">
-        <v>2782.955559373141</v>
-      </c>
-      <c r="M286" t="n">
-        <v>2607.085011948757</v>
-      </c>
-      <c r="N286" t="n">
-        <v>83.98837288254001</v>
-      </c>
-      <c r="O286" t="n">
-        <v>2384.207646674</v>
-      </c>
-      <c r="P286" t="n">
-        <v>4921.03817688</v>
-      </c>
-      <c r="Q286" t="n">
-        <v>1242.01</v>
-      </c>
-      <c r="R286" t="n">
-        <v>1542.52</v>
-      </c>
-      <c r="S286" t="n">
-        <v>350.0350000000004</v>
-      </c>
-      <c r="T286" t="n">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="287">
-      <c r="A287" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="B287" t="n">
-        <v>10000</v>
-      </c>
-      <c r="C287" t="n">
-        <v>2</v>
-      </c>
-      <c r="D287" t="n">
-        <v>1.570661462759655</v>
-      </c>
-      <c r="E287" t="n">
-        <v>9.591210385276415</v>
-      </c>
-      <c r="F287" t="n">
-        <v>14</v>
-      </c>
-      <c r="G287" t="n">
-        <v>7630.292013796412</v>
-      </c>
-      <c r="H287" t="n">
-        <v>0.08710379011183118</v>
-      </c>
-      <c r="I287" t="n">
-        <v>14</v>
-      </c>
-      <c r="J287" t="n">
-        <v>23.15734126984127</v>
-      </c>
-      <c r="K287" t="n">
-        <v>3997.56</v>
-      </c>
-      <c r="L287" t="n">
-        <v>15629.01998012371</v>
-      </c>
-      <c r="M287" t="n">
-        <v>6487.550128401559</v>
-      </c>
-      <c r="N287" t="n">
-        <v>741.7082303399999</v>
-      </c>
-      <c r="O287" t="n">
-        <v>7106.6838794</v>
-      </c>
-      <c r="P287" t="n">
-        <v>28533.419418</v>
-      </c>
-      <c r="Q287" t="n">
-        <v>1242.01</v>
-      </c>
-      <c r="R287" t="n">
-        <v>1542.52</v>
-      </c>
-      <c r="S287" t="n">
-        <v>350.0350000000004</v>
-      </c>
-      <c r="T287" t="n">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="288">
-      <c r="A288" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="B288" t="n">
-        <v>5000</v>
-      </c>
-      <c r="C288" t="n">
-        <v>6</v>
-      </c>
-      <c r="D288" t="n">
-        <v>3.287455501299847</v>
-      </c>
-      <c r="E288" t="n">
-        <v>9.293565808940587</v>
-      </c>
-      <c r="F288" t="n">
-        <v>14</v>
-      </c>
-      <c r="G288" t="n">
-        <v>7630.292013796412</v>
-      </c>
-      <c r="H288" t="n">
-        <v>0.1742075802236624</v>
-      </c>
-      <c r="I288" t="n">
-        <v>14</v>
-      </c>
-      <c r="J288" t="n">
-        <v>23.15734126984127</v>
-      </c>
-      <c r="K288" t="n">
-        <v>2891.56</v>
-      </c>
-      <c r="L288" t="n">
-        <v>11761.96926324595</v>
-      </c>
-      <c r="M288" t="n">
-        <v>5319.413731221542</v>
-      </c>
-      <c r="N288" t="n">
-        <v>374.4457123995</v>
-      </c>
-      <c r="O288" t="n">
-        <v>4606.35457485</v>
-      </c>
-      <c r="P288" t="n">
-        <v>16031.772862</v>
-      </c>
-      <c r="Q288" t="n">
-        <v>1242.01</v>
-      </c>
-      <c r="R288" t="n">
-        <v>1542.52</v>
-      </c>
-      <c r="S288" t="n">
-        <v>350.0350000000004</v>
-      </c>
-      <c r="T288" t="n">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="289">
-      <c r="A289" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="B289" t="n">
-        <v>5000</v>
-      </c>
-      <c r="C289" t="n">
-        <v>2</v>
-      </c>
-      <c r="D289" t="n">
-        <v>1.095818500433282</v>
-      </c>
-      <c r="E289" t="n">
-        <v>9.293565808940587</v>
-      </c>
-      <c r="F289" t="n">
-        <v>14</v>
-      </c>
-      <c r="G289" t="n">
-        <v>7630.292013796412</v>
-      </c>
-      <c r="H289" t="n">
-        <v>0.1742075802236624</v>
-      </c>
-      <c r="I289" t="n">
-        <v>14</v>
-      </c>
-      <c r="J289" t="n">
-        <v>23.15734126984127</v>
-      </c>
-      <c r="K289" t="n">
-        <v>2891.56</v>
-      </c>
-      <c r="L289" t="n">
-        <v>11761.96926324595</v>
-      </c>
-      <c r="M289" t="n">
-        <v>5319.413731221542</v>
-      </c>
-      <c r="N289" t="n">
-        <v>374.4457123995</v>
-      </c>
-      <c r="O289" t="n">
-        <v>4606.35457485</v>
-      </c>
-      <c r="P289" t="n">
-        <v>16031.772862</v>
-      </c>
-      <c r="Q289" t="n">
-        <v>1242.01</v>
-      </c>
-      <c r="R289" t="n">
-        <v>1542.52</v>
-      </c>
-      <c r="S289" t="n">
-        <v>350.0350000000004</v>
-      </c>
-      <c r="T289" t="n">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="290">
-      <c r="A290" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="B290" t="n">
-        <v>10000</v>
-      </c>
-      <c r="C290" t="n">
-        <v>6</v>
-      </c>
-      <c r="D290" t="n">
-        <v>4.711984388278966</v>
-      </c>
-      <c r="E290" t="n">
-        <v>9.591210385276415</v>
-      </c>
-      <c r="F290" t="n">
-        <v>14</v>
-      </c>
-      <c r="G290" t="n">
-        <v>7630.292013796412</v>
-      </c>
-      <c r="H290" t="n">
-        <v>0.08710379011183118</v>
-      </c>
-      <c r="I290" t="n">
-        <v>14</v>
-      </c>
-      <c r="J290" t="n">
-        <v>23.15734126984127</v>
-      </c>
-      <c r="K290" t="n">
-        <v>3997.56</v>
-      </c>
-      <c r="L290" t="n">
-        <v>15629.01998012371</v>
-      </c>
-      <c r="M290" t="n">
-        <v>6487.550128401559</v>
-      </c>
-      <c r="N290" t="n">
-        <v>741.7082303399999</v>
-      </c>
-      <c r="O290" t="n">
-        <v>7106.6838794</v>
-      </c>
-      <c r="P290" t="n">
-        <v>28533.419418</v>
-      </c>
-      <c r="Q290" t="n">
-        <v>1242.01</v>
-      </c>
-      <c r="R290" t="n">
-        <v>1542.52</v>
-      </c>
-      <c r="S290" t="n">
-        <v>350.0350000000004</v>
-      </c>
-      <c r="T290" t="n">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="291">
-      <c r="A291" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="B291" t="n">
-        <v>10000</v>
-      </c>
-      <c r="C291" t="n">
-        <v>4</v>
-      </c>
-      <c r="D291" t="n">
-        <v>3.141322925519311</v>
-      </c>
-      <c r="E291" t="n">
-        <v>9.591210385276415</v>
-      </c>
-      <c r="F291" t="n">
-        <v>14</v>
-      </c>
-      <c r="G291" t="n">
-        <v>7630.292013796412</v>
-      </c>
-      <c r="H291" t="n">
-        <v>0.08710379011183118</v>
-      </c>
-      <c r="I291" t="n">
-        <v>14</v>
-      </c>
-      <c r="J291" t="n">
-        <v>23.15734126984127</v>
-      </c>
-      <c r="K291" t="n">
-        <v>3997.56</v>
-      </c>
-      <c r="L291" t="n">
-        <v>15629.01998012371</v>
-      </c>
-      <c r="M291" t="n">
-        <v>6487.550128401559</v>
-      </c>
-      <c r="N291" t="n">
-        <v>741.7082303399999</v>
-      </c>
-      <c r="O291" t="n">
-        <v>7106.6838794</v>
-      </c>
-      <c r="P291" t="n">
-        <v>28533.419418</v>
-      </c>
-      <c r="Q291" t="n">
-        <v>1242.01</v>
-      </c>
-      <c r="R291" t="n">
-        <v>1542.52</v>
-      </c>
-      <c r="S291" t="n">
-        <v>350.0350000000004</v>
-      </c>
-      <c r="T291" t="n">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="292">
-      <c r="A292" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="B292" t="n">
-        <v>1000</v>
-      </c>
-      <c r="C292" t="n">
-        <v>10</v>
-      </c>
-      <c r="D292" t="n">
-        <v>1.619426228628243</v>
-      </c>
-      <c r="E292" t="n">
-        <v>9.856935437888509</v>
-      </c>
-      <c r="F292" t="n">
-        <v>14</v>
-      </c>
-      <c r="G292" t="n">
-        <v>7630.292013796412</v>
-      </c>
-      <c r="H292" t="n">
-        <v>0.8710379011183119</v>
-      </c>
-      <c r="I292" t="n">
-        <v>14</v>
-      </c>
-      <c r="J292" t="n">
-        <v>23.15734126984127</v>
-      </c>
-      <c r="K292" t="n">
-        <v>2006.76</v>
-      </c>
-      <c r="L292" t="n">
-        <v>2782.955559373141</v>
-      </c>
-      <c r="M292" t="n">
-        <v>2607.085011948757</v>
-      </c>
-      <c r="N292" t="n">
-        <v>83.98837288254001</v>
-      </c>
-      <c r="O292" t="n">
-        <v>2384.207646674</v>
-      </c>
-      <c r="P292" t="n">
-        <v>4921.03817688</v>
-      </c>
-      <c r="Q292" t="n">
-        <v>1242.01</v>
-      </c>
-      <c r="R292" t="n">
-        <v>1542.52</v>
-      </c>
-      <c r="S292" t="n">
-        <v>350.0350000000004</v>
-      </c>
-      <c r="T292" t="n">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="293">
-      <c r="A293" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="B293" t="n">
-        <v>10000</v>
-      </c>
-      <c r="C293" t="n">
-        <v>14</v>
-      </c>
-      <c r="D293" t="n">
-        <v>10.99463023931759</v>
-      </c>
-      <c r="E293" t="n">
-        <v>9.591210385276415</v>
-      </c>
-      <c r="F293" t="n">
-        <v>14</v>
-      </c>
-      <c r="G293" t="n">
-        <v>7630.292013796412</v>
-      </c>
-      <c r="H293" t="n">
-        <v>0.08710379011183118</v>
-      </c>
-      <c r="I293" t="n">
-        <v>14</v>
-      </c>
-      <c r="J293" t="n">
-        <v>23.15734126984127</v>
-      </c>
-      <c r="K293" t="n">
-        <v>3997.56</v>
-      </c>
-      <c r="L293" t="n">
-        <v>15629.01998012371</v>
-      </c>
-      <c r="M293" t="n">
-        <v>6487.550128401559</v>
-      </c>
-      <c r="N293" t="n">
-        <v>741.7082303399999</v>
-      </c>
-      <c r="O293" t="n">
-        <v>7106.6838794</v>
-      </c>
-      <c r="P293" t="n">
-        <v>28533.419418</v>
-      </c>
-      <c r="Q293" t="n">
-        <v>1242.01</v>
-      </c>
-      <c r="R293" t="n">
-        <v>1542.52</v>
-      </c>
-      <c r="S293" t="n">
-        <v>350.0350000000004</v>
-      </c>
-      <c r="T293" t="n">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="294">
-      <c r="A294" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="B294" t="n">
-        <v>5000</v>
-      </c>
-      <c r="C294" t="n">
-        <v>14</v>
-      </c>
-      <c r="D294" t="n">
-        <v>7.670729503032977</v>
-      </c>
-      <c r="E294" t="n">
-        <v>9.293565808940587</v>
-      </c>
-      <c r="F294" t="n">
-        <v>14</v>
-      </c>
-      <c r="G294" t="n">
-        <v>7630.292013796412</v>
-      </c>
-      <c r="H294" t="n">
-        <v>0.1742075802236624</v>
-      </c>
-      <c r="I294" t="n">
-        <v>14</v>
-      </c>
-      <c r="J294" t="n">
-        <v>23.15734126984127</v>
-      </c>
-      <c r="K294" t="n">
-        <v>2891.56</v>
-      </c>
-      <c r="L294" t="n">
-        <v>11761.96926324595</v>
-      </c>
-      <c r="M294" t="n">
-        <v>5319.413731221542</v>
-      </c>
-      <c r="N294" t="n">
-        <v>374.4457123995</v>
-      </c>
-      <c r="O294" t="n">
-        <v>4606.35457485</v>
-      </c>
-      <c r="P294" t="n">
-        <v>16031.772862</v>
-      </c>
-      <c r="Q294" t="n">
-        <v>1242.01</v>
-      </c>
-      <c r="R294" t="n">
-        <v>1542.52</v>
-      </c>
-      <c r="S294" t="n">
-        <v>350.0350000000004</v>
-      </c>
-      <c r="T294" t="n">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="295">
-      <c r="A295" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="B295" t="n">
-        <v>20000</v>
-      </c>
-      <c r="C295" t="n">
-        <v>2</v>
-      </c>
-      <c r="D295" t="n">
-        <v>1.856513018878587</v>
-      </c>
-      <c r="E295" t="n">
-        <v>10.0402636072274</v>
-      </c>
-      <c r="F295" t="n">
-        <v>14</v>
-      </c>
-      <c r="G295" t="n">
-        <v>7630.292013796412</v>
-      </c>
-      <c r="H295" t="n">
-        <v>0.04355189505591559</v>
-      </c>
-      <c r="I295" t="n">
-        <v>14</v>
-      </c>
-      <c r="J295" t="n">
-        <v>23.15734126984127</v>
-      </c>
-      <c r="K295" t="n">
-        <v>6209.560000000001</v>
-      </c>
-      <c r="L295" t="n">
-        <v>19496.07069700147</v>
-      </c>
-      <c r="M295" t="n">
-        <v>7655.686525581573</v>
-      </c>
-      <c r="N295" t="n">
-        <v>1490.202744702</v>
-      </c>
-      <c r="O295" t="n">
-        <v>11182.8279696</v>
-      </c>
-      <c r="P295" t="n">
-        <v>48914.13986199999</v>
-      </c>
-      <c r="Q295" t="n">
-        <v>1242.01</v>
-      </c>
-      <c r="R295" t="n">
-        <v>1542.52</v>
-      </c>
-      <c r="S295" t="n">
-        <v>350.0350000000004</v>
-      </c>
-      <c r="T295" t="n">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="296">
-      <c r="A296" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="B296" t="n">
-        <v>20000</v>
-      </c>
-      <c r="C296" t="n">
-        <v>6</v>
-      </c>
-      <c r="D296" t="n">
-        <v>5.569539056635763</v>
-      </c>
-      <c r="E296" t="n">
-        <v>10.0402636072274</v>
-      </c>
-      <c r="F296" t="n">
-        <v>14</v>
-      </c>
-      <c r="G296" t="n">
-        <v>7630.292013796412</v>
-      </c>
-      <c r="H296" t="n">
-        <v>0.04355189505591559</v>
-      </c>
-      <c r="I296" t="n">
-        <v>14</v>
-      </c>
-      <c r="J296" t="n">
-        <v>23.15734126984127</v>
-      </c>
-      <c r="K296" t="n">
-        <v>6209.560000000001</v>
-      </c>
-      <c r="L296" t="n">
-        <v>19496.07069700147</v>
-      </c>
-      <c r="M296" t="n">
-        <v>7655.686525581573</v>
-      </c>
-      <c r="N296" t="n">
-        <v>1490.202744702</v>
-      </c>
-      <c r="O296" t="n">
-        <v>11182.8279696</v>
-      </c>
-      <c r="P296" t="n">
-        <v>48914.13986199999</v>
-      </c>
-      <c r="Q296" t="n">
-        <v>1242.01</v>
-      </c>
-      <c r="R296" t="n">
-        <v>1542.52</v>
-      </c>
-      <c r="S296" t="n">
-        <v>350.0350000000004</v>
-      </c>
-      <c r="T296" t="n">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="297">
-      <c r="A297" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="B297" t="n">
-        <v>5000</v>
-      </c>
-      <c r="C297" t="n">
-        <v>10</v>
-      </c>
-      <c r="D297" t="n">
-        <v>5.479092502166411</v>
-      </c>
-      <c r="E297" t="n">
-        <v>9.293565808940587</v>
-      </c>
-      <c r="F297" t="n">
-        <v>14</v>
-      </c>
-      <c r="G297" t="n">
-        <v>7630.292013796412</v>
-      </c>
-      <c r="H297" t="n">
-        <v>0.1742075802236624</v>
-      </c>
-      <c r="I297" t="n">
-        <v>14</v>
-      </c>
-      <c r="J297" t="n">
-        <v>23.15734126984127</v>
-      </c>
-      <c r="K297" t="n">
-        <v>2891.56</v>
-      </c>
-      <c r="L297" t="n">
-        <v>11761.96926324595</v>
-      </c>
-      <c r="M297" t="n">
-        <v>5319.413731221542</v>
-      </c>
-      <c r="N297" t="n">
-        <v>374.4457123995</v>
-      </c>
-      <c r="O297" t="n">
-        <v>4606.35457485</v>
-      </c>
-      <c r="P297" t="n">
-        <v>16031.772862</v>
-      </c>
-      <c r="Q297" t="n">
-        <v>1242.01</v>
-      </c>
-      <c r="R297" t="n">
-        <v>1542.52</v>
-      </c>
-      <c r="S297" t="n">
-        <v>350.0350000000004</v>
-      </c>
-      <c r="T297" t="n">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="298">
-      <c r="A298" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="B298" t="n">
-        <v>20000</v>
-      </c>
-      <c r="C298" t="n">
-        <v>4</v>
-      </c>
-      <c r="D298" t="n">
-        <v>3.713026037757175</v>
-      </c>
-      <c r="E298" t="n">
-        <v>10.0402636072274</v>
-      </c>
-      <c r="F298" t="n">
-        <v>14</v>
-      </c>
-      <c r="G298" t="n">
-        <v>7630.292013796412</v>
-      </c>
-      <c r="H298" t="n">
-        <v>0.04355189505591559</v>
-      </c>
-      <c r="I298" t="n">
-        <v>14</v>
-      </c>
-      <c r="J298" t="n">
-        <v>23.15734126984127</v>
-      </c>
-      <c r="K298" t="n">
-        <v>6209.560000000001</v>
-      </c>
-      <c r="L298" t="n">
-        <v>19496.07069700147</v>
-      </c>
-      <c r="M298" t="n">
-        <v>7655.686525581573</v>
-      </c>
-      <c r="N298" t="n">
-        <v>1490.202744702</v>
-      </c>
-      <c r="O298" t="n">
-        <v>11182.8279696</v>
-      </c>
-      <c r="P298" t="n">
-        <v>48914.13986199999</v>
-      </c>
-      <c r="Q298" t="n">
-        <v>1242.01</v>
-      </c>
-      <c r="R298" t="n">
-        <v>1542.52</v>
-      </c>
-      <c r="S298" t="n">
-        <v>350.0350000000004</v>
-      </c>
-      <c r="T298" t="n">
-        <v>3000</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>